<commit_message>
ci(dev): publish dev build from 0e739b260a31ffd086530e217973248c6535c420 0e739b260a31ffd086530e217973248c6535c420
</commit_message>
<xml_diff>
--- a/dev/CodeSystem-PHFDACPRCS.xlsx
+++ b/dev/CodeSystem-PHFDACPRCS.xlsx
@@ -25,7 +25,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://verification.fda.gov.ph/</t>
+    <t>https://verification.fda.gov.ph</t>
   </si>
   <si>
     <t>Version</t>
@@ -79,7 +79,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>Philippines</t>
+    <t>Philippines (the)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>